<commit_message>
Extend monitoring coverage for the TMS rules and scenarios catalogue
- End-of-day wallet balance ingestion and balance aggregates/fields
- Multi-hop chain aggregate (layering) and peer percentile by segment
- Industry benchmarks (benchmarkDeviation) and invoice/trade fields
- Thresholds by attribute (valueBy), maintained lookup lists (inList)
- Household subject and cash transaction reports (CTR) workflow
- UI pages, tests (31 coverage checks, 16 newly executable workbook cases), docs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118Z57tGVFau2NaQGWr5ycA
</commit_message>
<xml_diff>
--- a/docs/test-results/AML_Transaction_Monitoring_Test_Cases_RESULTS.xlsx
+++ b/docs/test-results/AML_Transaction_Monitoring_Test_Cases_RESULTS.xlsx
@@ -7088,7 +7088,7 @@
       </c>
       <c r="K2" s="29" t="inlineStr">
         <is>
-          <t>1 alert (ALR-202610-000146) triggered by the 20th withdrawal (V01A-369-19); 20 contributing transactions linked; evidence window 2025-01-03 21:00Z–2025-01-04 21:00Z.</t>
+          <t>1 alert (ALR-202610-000182) triggered by the 20th withdrawal (V01A-522-19); 20 contributing transactions linked; evidence window 2025-01-03 21:00Z–2025-01-04 21:00Z.</t>
         </is>
       </c>
       <c r="L2" s="29" t="inlineStr">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="M2" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N2" s="29" t="n"/>
@@ -7171,7 +7171,7 @@
       </c>
       <c r="M3" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N3" s="29" t="n"/>
@@ -7244,7 +7244,7 @@
       </c>
       <c r="M4" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N4" s="29" t="n"/>
@@ -7317,7 +7317,7 @@
       </c>
       <c r="M5" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N5" s="29" t="n"/>
@@ -7390,7 +7390,7 @@
       </c>
       <c r="M6" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N6" s="29" t="n"/>
@@ -7463,7 +7463,7 @@
       </c>
       <c r="M7" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N7" s="29" t="n"/>
@@ -7536,7 +7536,7 @@
       </c>
       <c r="M8" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N8" s="29" t="n"/>
@@ -7609,7 +7609,7 @@
       </c>
       <c r="M9" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N9" s="29" t="n"/>
@@ -7682,7 +7682,7 @@
       </c>
       <c r="M10" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N10" s="29" t="n"/>
@@ -7755,7 +7755,7 @@
       </c>
       <c r="M11" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N11" s="29" t="n"/>
@@ -7828,7 +7828,7 @@
       </c>
       <c r="M12" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N12" s="29" t="n"/>
@@ -7901,7 +7901,7 @@
       </c>
       <c r="M13" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N13" s="29" t="n"/>
@@ -7974,7 +7974,7 @@
       </c>
       <c r="M14" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N14" s="29" t="n"/>
@@ -8047,7 +8047,7 @@
       </c>
       <c r="M15" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N15" s="29" t="inlineStr">
@@ -8057,7 +8057,7 @@
       </c>
       <c r="O15" s="29" t="inlineStr">
         <is>
-          <t>Automated: VelocityTests.VEL_03_outgoing_p2p_per_day. Failed in the first execution (DEF-TM-01: Own-wallet / self-transfer exclusion not configurable); fixed: Rule field txn.isOwnAccount; re-tested 2026-10-15.</t>
+          <t>Automated: VelocityTests.VEL_03_outgoing_p2p_per_day. Failed in the first execution (DEF-TM-01: Own-wallet / self-transfer exclusion not configurable); fixed: Rule field txn.isOwnAccount; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -8124,7 +8124,7 @@
       </c>
       <c r="M16" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N16" s="29" t="n"/>
@@ -8197,7 +8197,7 @@
       </c>
       <c r="M17" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N17" s="29" t="n"/>
@@ -8270,7 +8270,7 @@
       </c>
       <c r="M18" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N18" s="29" t="n"/>
@@ -8343,7 +8343,7 @@
       </c>
       <c r="M19" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N19" s="29" t="n"/>
@@ -8416,7 +8416,7 @@
       </c>
       <c r="M20" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N20" s="29" t="n"/>
@@ -8489,7 +8489,7 @@
       </c>
       <c r="M21" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N21" s="29" t="n"/>
@@ -8562,7 +8562,7 @@
       </c>
       <c r="M22" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N22" s="29" t="n"/>
@@ -8635,7 +8635,7 @@
       </c>
       <c r="M23" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N23" s="29" t="n"/>
@@ -8708,7 +8708,7 @@
       </c>
       <c r="M24" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N24" s="29" t="n"/>
@@ -8781,7 +8781,7 @@
       </c>
       <c r="M25" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N25" s="29" t="n"/>
@@ -8854,7 +8854,7 @@
       </c>
       <c r="M26" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N26" s="29" t="n"/>
@@ -8927,7 +8927,7 @@
       </c>
       <c r="M27" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N27" s="29" t="n"/>
@@ -8990,7 +8990,7 @@
       </c>
       <c r="K28" s="29" t="inlineStr">
         <is>
-          <t>Registration date missing → no silent pass: condition not met and data-quality item "[R_9215E93CF89D/customer.accountAgeDays] Rule R_9215E93CF89D v1 could not evaluate 'customer.accountAgeDays' for customer 105: value missing; condition treated as not met (result incomplete). Complete the customer data.".</t>
+          <t>Registration date missing → no silent pass: condition not met and data-quality item "[R_91328C8C7C12/customer.accountAgeDays] Rule R_91328C8C7C12 v1 could not evaluate 'customer.accountAgeDays' for customer 258: value missing; condition treated as not met (result incomplete). Complete the customer data.".</t>
         </is>
       </c>
       <c r="L28" s="29" t="inlineStr">
@@ -9000,7 +9000,7 @@
       </c>
       <c r="M28" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N28" s="29" t="n"/>
@@ -9063,7 +9063,7 @@
       </c>
       <c r="K29" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L29" s="29" t="inlineStr">
@@ -9073,7 +9073,7 @@
       </c>
       <c r="M29" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N29" s="29" t="inlineStr">
@@ -9140,7 +9140,7 @@
       </c>
       <c r="K30" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L30" s="29" t="inlineStr">
@@ -9150,7 +9150,7 @@
       </c>
       <c r="M30" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N30" s="29" t="inlineStr">
@@ -9217,7 +9217,7 @@
       </c>
       <c r="K31" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L31" s="29" t="inlineStr">
@@ -9227,7 +9227,7 @@
       </c>
       <c r="M31" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N31" s="29" t="inlineStr">
@@ -9294,7 +9294,7 @@
       </c>
       <c r="K32" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L32" s="29" t="inlineStr">
@@ -9304,7 +9304,7 @@
       </c>
       <c r="M32" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N32" s="29" t="inlineStr">
@@ -9381,7 +9381,7 @@
       </c>
       <c r="M33" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N33" s="29" t="n"/>
@@ -9454,7 +9454,7 @@
       </c>
       <c r="M34" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N34" s="29" t="n"/>
@@ -9527,7 +9527,7 @@
       </c>
       <c r="M35" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N35" s="29" t="n"/>
@@ -9600,7 +9600,7 @@
       </c>
       <c r="M36" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N36" s="29" t="n"/>
@@ -9673,7 +9673,7 @@
       </c>
       <c r="M37" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N37" s="29" t="n"/>
@@ -9746,7 +9746,7 @@
       </c>
       <c r="M38" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N38" s="29" t="n"/>
@@ -9819,7 +9819,7 @@
       </c>
       <c r="M39" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N39" s="29" t="n"/>
@@ -9892,7 +9892,7 @@
       </c>
       <c r="M40" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N40" s="29" t="n"/>
@@ -9965,7 +9965,7 @@
       </c>
       <c r="M41" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N41" s="29" t="n"/>
@@ -10038,7 +10038,7 @@
       </c>
       <c r="M42" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N42" s="29" t="n"/>
@@ -10111,7 +10111,7 @@
       </c>
       <c r="M43" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N43" s="29" t="n"/>
@@ -10184,7 +10184,7 @@
       </c>
       <c r="M44" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N44" s="29" t="n"/>
@@ -10257,7 +10257,7 @@
       </c>
       <c r="M45" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N45" s="29" t="n"/>
@@ -10330,7 +10330,7 @@
       </c>
       <c r="M46" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N46" s="29" t="n"/>
@@ -10403,7 +10403,7 @@
       </c>
       <c r="M47" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N47" s="29" t="n"/>
@@ -10466,7 +10466,7 @@
       </c>
       <c r="K48" s="29" t="inlineStr">
         <is>
-          <t>Declared income missing → 0 alerts; condition treated as not met and data-quality item raised: "[R_9D2264D830AF/profile.declaredMonthlyIncome] Rule R_9D2264D830AF v1 could not evaluate 'profile.declaredMonthlyIncome' for customer 404: value missing; condition treated as not met (result incomplete). Complete the customer data." (execution status Succeeded).</t>
+          <t>Declared income missing → 0 alerts; condition treated as not met and data-quality item raised: "[R_E45C19AE3223/profile.declaredMonthlyIncome] Rule R_E45C19AE3223 v1 could not evaluate 'profile.declaredMonthlyIncome' for customer 557: value missing; condition treated as not met (result incomplete). Complete the customer data." (execution status Succeeded).</t>
         </is>
       </c>
       <c r="L48" s="29" t="inlineStr">
@@ -10476,7 +10476,7 @@
       </c>
       <c r="M48" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N48" s="29" t="inlineStr">
@@ -10486,7 +10486,7 @@
       </c>
       <c r="O48" s="29" t="inlineStr">
         <is>
-          <t>Automated: AmountTests.AMT_03_monthly_income_multiple. Failed in the first execution (DEF-TM-02: Missing profile/attribute data silently evaluated as no-match); fixed: Missing inputs raise RuleInputMissing data-quality items (result incomplete); re-tested 2026-10-15.</t>
+          <t>Automated: AmountTests.AMT_03_monthly_income_multiple. Failed in the first execution (DEF-TM-02: Missing profile/attribute data silently evaluated as no-match); fixed: Missing inputs raise RuleInputMissing data-quality items (result incomplete); re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -10553,7 +10553,7 @@
       </c>
       <c r="M49" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N49" s="29" t="n"/>
@@ -10626,7 +10626,7 @@
       </c>
       <c r="M50" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N50" s="29" t="n"/>
@@ -10699,7 +10699,7 @@
       </c>
       <c r="M51" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N51" s="29" t="n"/>
@@ -10772,7 +10772,7 @@
       </c>
       <c r="M52" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N52" s="29" t="n"/>
@@ -10845,7 +10845,7 @@
       </c>
       <c r="M53" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N53" s="29" t="n"/>
@@ -10918,7 +10918,7 @@
       </c>
       <c r="M54" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N54" s="29" t="n"/>
@@ -10991,7 +10991,7 @@
       </c>
       <c r="M55" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N55" s="29" t="n"/>
@@ -11064,7 +11064,7 @@
       </c>
       <c r="M56" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N56" s="29" t="n"/>
@@ -11137,7 +11137,7 @@
       </c>
       <c r="M57" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N57" s="29" t="n"/>
@@ -11193,14 +11193,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J58" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J58" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K58" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — peerRatio compares with the peer median of agent-processed volume only; no percentile, segment or minimum peer-group size. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerPercentile'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Student customer above all 60 peers of its segment (same type, occupation, region) → percentile 100 → 1 alert; peer count 60, median 395.0000 and P90 640.0000 in the evidence.</t>
         </is>
       </c>
       <c r="L58" s="29" t="inlineStr">
@@ -11210,17 +11210,13 @@
       </c>
       <c r="M58" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N58" s="29" t="inlineStr">
-        <is>
-          <t>GAP-AMT-06</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N58" s="29" t="n"/>
       <c r="O58" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.AMT_06_peer_group_percentile. Note: percentile = share of peers strictly below the customer, so 99.5 and 100 both satisfy P = 99.. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -11270,14 +11266,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J59" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J59" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K59" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — peerRatio compares with the peer median of agent-processed volume only; no percentile, segment or minimum peer-group size. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerPercentile'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Customer with 57 of 60 peers below (95th percentile) → 0 alerts.</t>
         </is>
       </c>
       <c r="L59" s="29" t="inlineStr">
@@ -11287,17 +11283,13 @@
       </c>
       <c r="M59" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N59" s="29" t="inlineStr">
-        <is>
-          <t>GAP-AMT-06</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N59" s="29" t="n"/>
       <c r="O59" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.AMT_06_peer_group_percentile. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -11347,14 +11339,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J60" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J60" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K60" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — peerRatio compares with the peer median of agent-processed volume only; no percentile, segment or minimum peer-group size. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerPercentile'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Peer group of 20 members (19 peers &lt; 50) → rule not evaluated for the customer (no alert) and logged as a RuleInputMissing data-quality item.</t>
         </is>
       </c>
       <c r="L60" s="29" t="inlineStr">
@@ -11364,17 +11356,13 @@
       </c>
       <c r="M60" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N60" s="29" t="inlineStr">
-        <is>
-          <t>GAP-AMT-06</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N60" s="29" t="n"/>
       <c r="O60" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.AMT_06_peer_group_percentile. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -11441,7 +11429,7 @@
       </c>
       <c r="M61" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N61" s="29" t="n"/>
@@ -11514,7 +11502,7 @@
       </c>
       <c r="M62" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N62" s="29" t="n"/>
@@ -11587,7 +11575,7 @@
       </c>
       <c r="M63" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N63" s="29" t="n"/>
@@ -11660,7 +11648,7 @@
       </c>
       <c r="M64" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N64" s="29" t="n"/>
@@ -11733,7 +11721,7 @@
       </c>
       <c r="M65" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N65" s="29" t="n"/>
@@ -11806,7 +11794,7 @@
       </c>
       <c r="M66" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N66" s="29" t="n"/>
@@ -11879,7 +11867,7 @@
       </c>
       <c r="M67" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N67" s="29" t="n"/>
@@ -11952,7 +11940,7 @@
       </c>
       <c r="M68" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N68" s="29" t="n"/>
@@ -12025,7 +12013,7 @@
       </c>
       <c r="M69" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N69" s="29" t="n"/>
@@ -12098,7 +12086,7 @@
       </c>
       <c r="M70" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N70" s="29" t="n"/>
@@ -12171,7 +12159,7 @@
       </c>
       <c r="M71" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N71" s="29" t="n"/>
@@ -12244,7 +12232,7 @@
       </c>
       <c r="M72" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N72" s="29" t="n"/>
@@ -12317,7 +12305,7 @@
       </c>
       <c r="M73" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N73" s="29" t="n"/>
@@ -12390,7 +12378,7 @@
       </c>
       <c r="M74" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N74" s="29" t="n"/>
@@ -12463,7 +12451,7 @@
       </c>
       <c r="M75" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N75" s="29" t="n"/>
@@ -12536,7 +12524,7 @@
       </c>
       <c r="M76" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N76" s="29" t="n"/>
@@ -12609,7 +12597,7 @@
       </c>
       <c r="M77" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N77" s="29" t="n"/>
@@ -12682,7 +12670,7 @@
       </c>
       <c r="M78" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N78" s="29" t="n"/>
@@ -12755,7 +12743,7 @@
       </c>
       <c r="M79" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N79" s="29" t="inlineStr">
@@ -12765,7 +12753,7 @@
       </c>
       <c r="O79" s="29" t="inlineStr">
         <is>
-          <t>Automated: StructuringTests.STR_03_smurfing. Failed in the first execution (DEF-TM-03: Entity-resolution links not usable by rules or shown in evidence); fixed: Subject 'Entity' (linked customers, minimum confidence) and linkedParties in alert evidence; re-tested 2026-10-15.</t>
+          <t>Automated: StructuringTests.STR_03_smurfing. Failed in the first execution (DEF-TM-03: Entity-resolution links not usable by rules or shown in evidence); fixed: Subject 'Entity' (linked customers, minimum confidence) and linkedParties in alert evidence; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -12832,7 +12820,7 @@
       </c>
       <c r="M80" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N80" s="29" t="n"/>
@@ -12905,7 +12893,7 @@
       </c>
       <c r="M81" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N81" s="29" t="n"/>
@@ -12978,7 +12966,7 @@
       </c>
       <c r="M82" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N82" s="29" t="inlineStr">
@@ -12988,7 +12976,7 @@
       </c>
       <c r="O82" s="29" t="inlineStr">
         <is>
-          <t>Automated: StructuringTests.STR_04_multiple_own_wallets. Failed in the first execution (DEF-TM-03: Entity-resolution links not usable by rules or shown in evidence); fixed: Subject 'Entity' (linked customers, minimum confidence) and linkedParties in alert evidence; re-tested 2026-10-15.</t>
+          <t>Automated: StructuringTests.STR_04_multiple_own_wallets. Failed in the first execution (DEF-TM-03: Entity-resolution links not usable by rules or shown in evidence); fixed: Subject 'Entity' (linked customers, minimum confidence) and linkedParties in alert evidence; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -13055,7 +13043,7 @@
       </c>
       <c r="M83" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N83" s="29" t="n"/>
@@ -13128,7 +13116,7 @@
       </c>
       <c r="M84" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N84" s="29" t="n"/>
@@ -13201,7 +13189,7 @@
       </c>
       <c r="M85" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N85" s="29" t="n"/>
@@ -13274,7 +13262,7 @@
       </c>
       <c r="M86" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N86" s="29" t="n"/>
@@ -13347,7 +13335,7 @@
       </c>
       <c r="M87" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N87" s="29" t="n"/>
@@ -13420,7 +13408,7 @@
       </c>
       <c r="M88" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N88" s="29" t="n"/>
@@ -13493,7 +13481,7 @@
       </c>
       <c r="M89" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N89" s="29" t="n"/>
@@ -13566,7 +13554,7 @@
       </c>
       <c r="M90" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N90" s="29" t="n"/>
@@ -13639,7 +13627,7 @@
       </c>
       <c r="M91" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N91" s="29" t="n"/>
@@ -13712,7 +13700,7 @@
       </c>
       <c r="M92" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N92" s="29" t="n"/>
@@ -13785,7 +13773,7 @@
       </c>
       <c r="M93" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N93" s="29" t="n"/>
@@ -13841,14 +13829,14 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J94" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J94" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K94" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Wallet balances / end-of-day balances are not ingested or available to rules. Closest rule definition rejected by the rule validator: $.condition.conditions[0].field: Unknown field 'wallet.endOfDayBalance': not present in the data-source registry..</t>
+          <t>Monthly in/out 6,000 with end-of-day balance between 2 and 4 → 1 alert (average balance and the daily balances in the evidence).</t>
         </is>
       </c>
       <c r="L94" s="29" t="inlineStr">
@@ -13858,17 +13846,13 @@
       </c>
       <c r="M94" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N94" s="29" t="inlineStr">
-        <is>
-          <t>GAP-RMV-02</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N94" s="29" t="n"/>
       <c r="O94" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.RMV_02_balance_kept_near_zero. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -13918,14 +13902,14 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J95" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J95" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K95" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Wallet balances / end-of-day balances are not ingested or available to rules. Closest rule definition rejected by the rule validator: $.condition.conditions[0].field: Unknown field 'wallet.endOfDayBalance': not present in the data-source registry..</t>
+          <t>Throughput 1,000 with the same balances → 0 alerts.</t>
         </is>
       </c>
       <c r="L95" s="29" t="inlineStr">
@@ -13935,17 +13919,13 @@
       </c>
       <c r="M95" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N95" s="29" t="inlineStr">
-        <is>
-          <t>GAP-RMV-02</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N95" s="29" t="n"/>
       <c r="O95" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.RMV_02_balance_kept_near_zero. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -13995,14 +13975,14 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J96" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J96" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K96" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Wallet balances / end-of-day balances are not ingested or available to rules. Closest rule definition rejected by the rule validator: $.condition.conditions[0].field: Unknown field 'wallet.endOfDayBalance': not present in the data-source registry..</t>
+          <t>Throughput 6,000 but no balance data from the core → 0 alerts; marked not evaluated with a RuleInputMissing data-quality item.</t>
         </is>
       </c>
       <c r="L96" s="29" t="inlineStr">
@@ -14012,17 +13992,13 @@
       </c>
       <c r="M96" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N96" s="29" t="inlineStr">
-        <is>
-          <t>GAP-RMV-02</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N96" s="29" t="n"/>
       <c r="O96" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.RMV_02_balance_kept_near_zero. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -14089,7 +14065,7 @@
       </c>
       <c r="M97" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N97" s="29" t="n"/>
@@ -14162,7 +14138,7 @@
       </c>
       <c r="M98" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N98" s="29" t="n"/>
@@ -14235,7 +14211,7 @@
       </c>
       <c r="M99" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N99" s="29" t="inlineStr">
@@ -14245,7 +14221,7 @@
       </c>
       <c r="O99" s="29" t="inlineStr">
         <is>
-          <t>Automated: RapidMovementFanTests.RMV_03_incoming_then_cash_out. Failed in the first execution (DEF-TM-04: No secondary indicator flags / severity escalation); fixed: action.indicators (flag + optional severity) and counterparty.* fields; re-tested 2026-10-15.</t>
+          <t>Automated: RapidMovementFanTests.RMV_03_incoming_then_cash_out. Failed in the first execution (DEF-TM-04: No secondary indicator flags / severity escalation); fixed: action.indicators (flag + optional severity) and counterparty.* fields; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -14295,14 +14271,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J100" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J100" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K100" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — cycle detects funds returning to the subject only; no open multi-hop chain (A→B→C→D) with per-hop retention. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'chain'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>A→B 1,000; B→C 950; C→D 920 within 6 hours (95 % / 97 % retained) → 1 alert on A with 3 hops in the evidence (B, C and D are alerted as chain members too).</t>
         </is>
       </c>
       <c r="L100" s="29" t="inlineStr">
@@ -14312,17 +14288,13 @@
       </c>
       <c r="M100" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N100" s="29" t="inlineStr">
-        <is>
-          <t>GAP-RMV-04</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N100" s="29" t="n"/>
       <c r="O100" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.RMV_04_layering_chain. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -14372,14 +14344,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J101" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J101" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K101" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — cycle detects funds returning to the subject only; no open multi-hop chain (A→B→C→D) with per-hop retention. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'chain'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Hops separated by 3 days → 0 alerts.</t>
         </is>
       </c>
       <c r="L101" s="29" t="inlineStr">
@@ -14389,17 +14361,13 @@
       </c>
       <c r="M101" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N101" s="29" t="inlineStr">
-        <is>
-          <t>GAP-RMV-04</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N101" s="29" t="n"/>
       <c r="O101" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.RMV_04_layering_chain. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -14449,14 +14417,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J102" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J102" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K102" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — cycle detects funds returning to the subject only; no open multi-hop chain (A→B→C→D) with per-hop retention. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'chain'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Only 2 hops → 0 alerts.</t>
         </is>
       </c>
       <c r="L102" s="29" t="inlineStr">
@@ -14466,17 +14434,13 @@
       </c>
       <c r="M102" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N102" s="29" t="inlineStr">
-        <is>
-          <t>GAP-RMV-04</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N102" s="29" t="n"/>
       <c r="O102" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.RMV_04_layering_chain. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -14526,14 +14490,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J103" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J103" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K103" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — cycle detects funds returning to the subject only; no open multi-hop chain (A→B→C→D) with per-hop retention. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'chain'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>One hop through internal clearing wallet: the two legs resolve to one economic transfer 96-&gt;97; clearing wallet skipped, chain still detected (1 alert).</t>
         </is>
       </c>
       <c r="L103" s="29" t="inlineStr">
@@ -14543,17 +14507,13 @@
       </c>
       <c r="M103" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N103" s="29" t="inlineStr">
-        <is>
-          <t>GAP-RMV-04</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N103" s="29" t="n"/>
       <c r="O103" s="29" t="inlineStr">
         <is>
-          <t>Automated: CapabilityGapTests.Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.RMV_04_layering_chain. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -14620,7 +14580,7 @@
       </c>
       <c r="M104" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N104" s="29" t="n"/>
@@ -14693,7 +14653,7 @@
       </c>
       <c r="M105" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N105" s="29" t="n"/>
@@ -14766,7 +14726,7 @@
       </c>
       <c r="M106" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N106" s="29" t="n"/>
@@ -14839,7 +14799,7 @@
       </c>
       <c r="M107" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N107" s="29" t="n"/>
@@ -14912,7 +14872,7 @@
       </c>
       <c r="M108" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N108" s="29" t="n"/>
@@ -14985,7 +14945,7 @@
       </c>
       <c r="M109" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N109" s="29" t="inlineStr">
@@ -14995,7 +14955,7 @@
       </c>
       <c r="O109" s="29" t="inlineStr">
         <is>
-          <t>Automated: RapidMovementFanTests.FAN_01_fan_in. Failed in the first execution (DEF-TM-04: No secondary indicator flags / severity escalation); fixed: action.indicators (flag + optional severity) and counterparty.* fields; re-tested 2026-10-15.</t>
+          <t>Automated: RapidMovementFanTests.FAN_01_fan_in. Failed in the first execution (DEF-TM-04: No secondary indicator flags / severity escalation); fixed: action.indicators (flag + optional severity) and counterparty.* fields; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -15062,7 +15022,7 @@
       </c>
       <c r="M110" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N110" s="29" t="n"/>
@@ -15135,7 +15095,7 @@
       </c>
       <c r="M111" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N111" s="29" t="n"/>
@@ -15208,7 +15168,7 @@
       </c>
       <c r="M112" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N112" s="29" t="n"/>
@@ -15281,7 +15241,7 @@
       </c>
       <c r="M113" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N113" s="29" t="inlineStr">
@@ -15291,7 +15251,7 @@
       </c>
       <c r="O113" s="29" t="inlineStr">
         <is>
-          <t>Automated: RapidMovementFanTests.FAN_02_fan_out. Failed in the first execution (DEF-TM-04: No secondary indicator flags / severity escalation); fixed: action.indicators (flag + optional severity) and counterparty.* fields; re-tested 2026-10-15.</t>
+          <t>Automated: RapidMovementFanTests.FAN_02_fan_out. Failed in the first execution (DEF-TM-04: No secondary indicator flags / severity escalation); fixed: action.indicators (flag + optional severity) and counterparty.* fields; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -15358,7 +15318,7 @@
       </c>
       <c r="M114" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N114" s="29" t="n"/>
@@ -15431,7 +15391,7 @@
       </c>
       <c r="M115" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N115" s="29" t="n"/>
@@ -15504,7 +15464,7 @@
       </c>
       <c r="M116" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N116" s="29" t="n"/>
@@ -15577,7 +15537,7 @@
       </c>
       <c r="M117" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N117" s="29" t="n"/>
@@ -15650,7 +15610,7 @@
       </c>
       <c r="M118" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N118" s="29" t="n"/>
@@ -15723,7 +15683,7 @@
       </c>
       <c r="M119" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N119" s="29" t="n"/>
@@ -15786,7 +15746,7 @@
       </c>
       <c r="K120" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L120" s="29" t="inlineStr">
@@ -15796,7 +15756,7 @@
       </c>
       <c r="M120" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N120" s="29" t="inlineStr">
@@ -15863,7 +15823,7 @@
       </c>
       <c r="K121" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L121" s="29" t="inlineStr">
@@ -15873,7 +15833,7 @@
       </c>
       <c r="M121" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N121" s="29" t="inlineStr">
@@ -15940,7 +15900,7 @@
       </c>
       <c r="K122" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L122" s="29" t="inlineStr">
@@ -15950,7 +15910,7 @@
       </c>
       <c r="M122" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N122" s="29" t="inlineStr">
@@ -16017,7 +15977,7 @@
       </c>
       <c r="K123" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L123" s="29" t="inlineStr">
@@ -16027,7 +15987,7 @@
       </c>
       <c r="M123" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N123" s="29" t="inlineStr">
@@ -16094,7 +16054,7 @@
       </c>
       <c r="K124" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L124" s="29" t="inlineStr">
@@ -16104,7 +16064,7 @@
       </c>
       <c r="M124" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N124" s="29" t="inlineStr">
@@ -16181,7 +16141,7 @@
       </c>
       <c r="M125" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N125" s="29" t="n"/>
@@ -16254,7 +16214,7 @@
       </c>
       <c r="M126" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N126" s="29" t="n"/>
@@ -16327,7 +16287,7 @@
       </c>
       <c r="M127" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N127" s="29" t="n"/>
@@ -16400,7 +16360,7 @@
       </c>
       <c r="M128" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N128" s="29" t="n"/>
@@ -16473,7 +16433,7 @@
       </c>
       <c r="M129" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N129" s="29" t="n"/>
@@ -16546,7 +16506,7 @@
       </c>
       <c r="M130" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N130" s="29" t="n"/>
@@ -16619,7 +16579,7 @@
       </c>
       <c r="M131" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N131" s="29" t="inlineStr">
@@ -16629,7 +16589,7 @@
       </c>
       <c r="O131" s="29" t="inlineStr">
         <is>
-          <t>Automated: GeographicTests.GEO_03_high_risk_jurisdiction. Failed in the first execution (DEF-TM-05: Runs used the active rule version for all transactions); fixed: Manual runs evaluate each period with the version in force at transaction time; re-tested 2026-10-15.</t>
+          <t>Automated: GeographicTests.GEO_03_high_risk_jurisdiction. Failed in the first execution (DEF-TM-05: Runs used the active rule version for all transactions); fixed: Manual runs evaluate each period with the version in force at transaction time; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -16696,7 +16656,7 @@
       </c>
       <c r="M132" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N132" s="29" t="n"/>
@@ -16769,7 +16729,7 @@
       </c>
       <c r="M133" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N133" s="29" t="n"/>
@@ -16842,7 +16802,7 @@
       </c>
       <c r="M134" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N134" s="29" t="n"/>
@@ -16915,7 +16875,7 @@
       </c>
       <c r="M135" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N135" s="29" t="n"/>
@@ -16988,7 +16948,7 @@
       </c>
       <c r="M136" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N136" s="29" t="n"/>
@@ -17061,7 +17021,7 @@
       </c>
       <c r="M137" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N137" s="29" t="n"/>
@@ -17134,7 +17094,7 @@
       </c>
       <c r="M138" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N138" s="29" t="n"/>
@@ -17207,7 +17167,7 @@
       </c>
       <c r="M139" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N139" s="29" t="n"/>
@@ -17270,7 +17230,7 @@
       </c>
       <c r="K140" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No 'first cross-border after M months domestic-only' aggregate (newCountries ignores amount and months of domestic history). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'firstCrossBorderAfterMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No 'first cross-border after M months domestic-only' aggregate (newCountries ignores amount and months of domestic history). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'firstCrossBorderAfterMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L140" s="29" t="inlineStr">
@@ -17280,7 +17240,7 @@
       </c>
       <c r="M140" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N140" s="29" t="inlineStr">
@@ -17347,7 +17307,7 @@
       </c>
       <c r="K141" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No 'first cross-border after M months domestic-only' aggregate (newCountries ignores amount and months of domestic history). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'firstCrossBorderAfterMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No 'first cross-border after M months domestic-only' aggregate (newCountries ignores amount and months of domestic history). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'firstCrossBorderAfterMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L141" s="29" t="inlineStr">
@@ -17357,7 +17317,7 @@
       </c>
       <c r="M141" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N141" s="29" t="inlineStr">
@@ -17424,7 +17384,7 @@
       </c>
       <c r="K142" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Agent locations / distances are not modelled; cash-in and cash-out by different persons cannot be correlated. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Agent locations / distances are not modelled; cash-in and cash-out by different persons cannot be correlated. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L142" s="29" t="inlineStr">
@@ -17434,7 +17394,7 @@
       </c>
       <c r="M142" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N142" s="29" t="inlineStr">
@@ -17501,7 +17461,7 @@
       </c>
       <c r="K143" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Agent locations / distances are not modelled; cash-in and cash-out by different persons cannot be correlated. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Agent locations / distances are not modelled; cash-in and cash-out by different persons cannot be correlated. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L143" s="29" t="inlineStr">
@@ -17511,7 +17471,7 @@
       </c>
       <c r="M143" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N143" s="29" t="inlineStr">
@@ -17588,7 +17548,7 @@
       </c>
       <c r="M144" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N144" s="29" t="inlineStr">
@@ -17665,7 +17625,7 @@
       </c>
       <c r="M145" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N145" s="29" t="inlineStr">
@@ -17742,7 +17702,7 @@
       </c>
       <c r="M146" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N146" s="29" t="n"/>
@@ -17815,7 +17775,7 @@
       </c>
       <c r="M147" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N147" s="29" t="n"/>
@@ -17888,7 +17848,7 @@
       </c>
       <c r="M148" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N148" s="29" t="n"/>
@@ -17961,7 +17921,7 @@
       </c>
       <c r="M149" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N149" s="29" t="n"/>
@@ -18034,7 +17994,7 @@
       </c>
       <c r="M150" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N150" s="29" t="n"/>
@@ -18107,7 +18067,7 @@
       </c>
       <c r="M151" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N151" s="29" t="n"/>
@@ -18180,7 +18140,7 @@
       </c>
       <c r="M152" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N152" s="29" t="inlineStr">
@@ -18257,7 +18217,7 @@
       </c>
       <c r="M153" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N153" s="29" t="inlineStr">
@@ -18334,7 +18294,7 @@
       </c>
       <c r="M154" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N154" s="29" t="inlineStr">
@@ -18411,7 +18371,7 @@
       </c>
       <c r="M155" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N155" s="29" t="inlineStr">
@@ -18488,7 +18448,7 @@
       </c>
       <c r="M156" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N156" s="29" t="n"/>
@@ -18561,7 +18521,7 @@
       </c>
       <c r="M157" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N157" s="29" t="n"/>
@@ -18634,7 +18594,7 @@
       </c>
       <c r="M158" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N158" s="29" t="n"/>
@@ -18707,7 +18667,7 @@
       </c>
       <c r="M159" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N159" s="29" t="n"/>
@@ -18770,7 +18730,7 @@
       </c>
       <c r="K160" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Channel limit-hit events are not ingested; channel switch sequence cannot be expressed. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'channelSwitchAfterLimit'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Channel limit-hit events are not ingested; channel switch sequence cannot be expressed. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'channelSwitchAfterLimit'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L160" s="29" t="inlineStr">
@@ -18780,7 +18740,7 @@
       </c>
       <c r="M160" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N160" s="29" t="inlineStr">
@@ -18847,7 +18807,7 @@
       </c>
       <c r="K161" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Channel limit-hit events are not ingested; channel switch sequence cannot be expressed. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'channelSwitchAfterLimit'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Channel limit-hit events are not ingested; channel switch sequence cannot be expressed. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'channelSwitchAfterLimit'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L161" s="29" t="inlineStr">
@@ -18857,7 +18817,7 @@
       </c>
       <c r="M161" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N161" s="29" t="inlineStr">
@@ -18934,7 +18894,7 @@
       </c>
       <c r="M162" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N162" s="29" t="n"/>
@@ -19007,7 +18967,7 @@
       </c>
       <c r="M163" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N163" s="29" t="n"/>
@@ -19080,7 +19040,7 @@
       </c>
       <c r="M164" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N164" s="29" t="n"/>
@@ -19153,7 +19113,7 @@
       </c>
       <c r="M165" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N165" s="29" t="n"/>
@@ -19226,7 +19186,7 @@
       </c>
       <c r="M166" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N166" s="29" t="n"/>
@@ -19299,7 +19259,7 @@
       </c>
       <c r="M167" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N167" s="29" t="n"/>
@@ -19372,7 +19332,7 @@
       </c>
       <c r="M168" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N168" s="29" t="n"/>
@@ -19445,7 +19405,7 @@
       </c>
       <c r="M169" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N169" s="29" t="inlineStr">
@@ -19455,7 +19415,7 @@
       </c>
       <c r="O169" s="29" t="inlineStr">
         <is>
-          <t>Automated: BehaviourTests.BEH_03_night_activity. Failed in the first execution (DEF-TM-06: No per-customer behavioural baseline); fixed: historyCount / historySum / historyRatio aggregates over the customer's own lookback; re-tested 2026-10-15.</t>
+          <t>Automated: BehaviourTests.BEH_03_night_activity. Failed in the first execution (DEF-TM-06: No per-customer behavioural baseline); fixed: historyCount / historySum / historyRatio aggregates over the customer's own lookback; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -19522,7 +19482,7 @@
       </c>
       <c r="M170" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N170" s="29" t="n"/>
@@ -19595,7 +19555,7 @@
       </c>
       <c r="M171" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N171" s="29" t="n"/>
@@ -19668,7 +19628,7 @@
       </c>
       <c r="M172" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N172" s="29" t="inlineStr">
@@ -19678,7 +19638,7 @@
       </c>
       <c r="O172" s="29" t="inlineStr">
         <is>
-          <t>Automated: BehaviourTests.BEH_04_occupation_mismatch. Failed in the first execution (DEF-TM-02: Missing profile/attribute data silently evaluated as no-match); fixed: Missing inputs raise RuleInputMissing data-quality items (result incomplete); re-tested 2026-10-15.</t>
+          <t>Automated: BehaviourTests.BEH_04_occupation_mismatch. Failed in the first execution (DEF-TM-02: Missing profile/attribute data silently evaluated as no-match); fixed: Missing inputs raise RuleInputMissing data-quality items (result incomplete); re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -19745,7 +19705,7 @@
       </c>
       <c r="M173" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N173" s="29" t="n"/>
@@ -19818,7 +19778,7 @@
       </c>
       <c r="M174" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N174" s="29" t="n"/>
@@ -19891,7 +19851,7 @@
       </c>
       <c r="M175" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N175" s="29" t="n"/>
@@ -19964,7 +19924,7 @@
       </c>
       <c r="M176" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N176" s="29" t="n"/>
@@ -20027,7 +19987,7 @@
       </c>
       <c r="K177" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No salary-credit linkage or 'M consecutive months' pattern. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'salaryRemittedShareConsecutiveMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No salary-credit linkage or 'M consecutive months' pattern. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'salaryRemittedShareConsecutiveMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L177" s="29" t="inlineStr">
@@ -20037,7 +19997,7 @@
       </c>
       <c r="M177" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N177" s="29" t="inlineStr">
@@ -20104,7 +20064,7 @@
       </c>
       <c r="K178" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No salary-credit linkage or 'M consecutive months' pattern. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'salaryRemittedShareConsecutiveMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No salary-credit linkage or 'M consecutive months' pattern. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'salaryRemittedShareConsecutiveMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L178" s="29" t="inlineStr">
@@ -20114,7 +20074,7 @@
       </c>
       <c r="M178" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N178" s="29" t="inlineStr">
@@ -20191,7 +20151,7 @@
       </c>
       <c r="M179" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N179" s="29" t="n"/>
@@ -20264,7 +20224,7 @@
       </c>
       <c r="M180" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N180" s="29" t="n"/>
@@ -20337,7 +20297,7 @@
       </c>
       <c r="M181" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N181" s="29" t="n"/>
@@ -20410,7 +20370,7 @@
       </c>
       <c r="M182" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N182" s="29" t="n"/>
@@ -20483,7 +20443,7 @@
       </c>
       <c r="M183" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N183" s="29" t="n"/>
@@ -20556,7 +20516,7 @@
       </c>
       <c r="M184" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N184" s="29" t="n"/>
@@ -20629,7 +20589,7 @@
       </c>
       <c r="M185" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N185" s="29" t="n"/>
@@ -20702,7 +20662,7 @@
       </c>
       <c r="M186" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N186" s="29" t="n"/>
@@ -20775,7 +20735,7 @@
       </c>
       <c r="M187" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N187" s="29" t="n"/>
@@ -20848,7 +20808,7 @@
       </c>
       <c r="M188" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N188" s="29" t="n"/>
@@ -20921,7 +20881,7 @@
       </c>
       <c r="M189" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N189" s="29" t="n"/>
@@ -20994,7 +20954,7 @@
       </c>
       <c r="M190" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N190" s="29" t="n"/>
@@ -21067,7 +21027,7 @@
       </c>
       <c r="M191" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N191" s="29" t="n"/>
@@ -21130,7 +21090,7 @@
       </c>
       <c r="K192" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Rules cannot test links between the agent and the customers it serves (shared ID/phone/device/family). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentLinkedCustomerTxns'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Rules cannot test links between the agent and the customers it serves (shared ID/phone/device/family). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentLinkedCustomerTxns'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L192" s="29" t="inlineStr">
@@ -21140,7 +21100,7 @@
       </c>
       <c r="M192" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N192" s="29" t="inlineStr">
@@ -21207,7 +21167,7 @@
       </c>
       <c r="K193" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Rules cannot test links between the agent and the customers it serves (shared ID/phone/device/family). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentLinkedCustomerTxns'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Rules cannot test links between the agent and the customers it serves (shared ID/phone/device/family). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentLinkedCustomerTxns'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L193" s="29" t="inlineStr">
@@ -21217,7 +21177,7 @@
       </c>
       <c r="M193" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N193" s="29" t="inlineStr">
@@ -21284,7 +21244,7 @@
       </c>
       <c r="K194" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — peerRatio uses agent volume, not the cash-out/cash-in ratio compared with a regional peer median × R. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerRatioOfRatio'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — peerRatio uses agent volume, not the cash-out/cash-in ratio compared with a regional peer median × R. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerRatioOfRatio'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L194" s="29" t="inlineStr">
@@ -21294,7 +21254,7 @@
       </c>
       <c r="M194" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N194" s="29" t="inlineStr">
@@ -21361,7 +21321,7 @@
       </c>
       <c r="K195" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — peerRatio uses agent volume, not the cash-out/cash-in ratio compared with a regional peer median × R. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerRatioOfRatio'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — peerRatio uses agent volume, not the cash-out/cash-in ratio compared with a regional peer median × R. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerRatioOfRatio'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L195" s="29" t="inlineStr">
@@ -21371,7 +21331,7 @@
       </c>
       <c r="M195" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N195" s="29" t="inlineStr">
@@ -21448,7 +21408,7 @@
       </c>
       <c r="M196" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N196" s="29" t="n"/>
@@ -21521,7 +21481,7 @@
       </c>
       <c r="M197" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N197" s="29" t="n"/>
@@ -21594,7 +21554,7 @@
       </c>
       <c r="M198" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N198" s="29" t="n"/>
@@ -21657,7 +21617,7 @@
       </c>
       <c r="K199" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No 'customers registered by agent who transact within 24 h' share aggregate. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentNewCustomerActiveShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No 'customers registered by agent who transact within 24 h' share aggregate. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentNewCustomerActiveShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L199" s="29" t="inlineStr">
@@ -21667,7 +21627,7 @@
       </c>
       <c r="M199" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N199" s="29" t="inlineStr">
@@ -21734,7 +21694,7 @@
       </c>
       <c r="K200" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No 'customers registered by agent who transact within 24 h' share aggregate. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentNewCustomerActiveShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No 'customers registered by agent who transact within 24 h' share aggregate. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentNewCustomerActiveShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L200" s="29" t="inlineStr">
@@ -21744,7 +21704,7 @@
       </c>
       <c r="M200" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N200" s="29" t="inlineStr">
@@ -21821,7 +21781,7 @@
       </c>
       <c r="M201" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N201" s="29" t="n"/>
@@ -21894,7 +21854,7 @@
       </c>
       <c r="M202" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N202" s="29" t="n"/>
@@ -21957,7 +21917,7 @@
       </c>
       <c r="K203" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Agent location / customer residence distance is not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Agent location / customer residence distance is not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L203" s="29" t="inlineStr">
@@ -21967,7 +21927,7 @@
       </c>
       <c r="M203" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N203" s="29" t="inlineStr">
@@ -22034,7 +21994,7 @@
       </c>
       <c r="K204" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Agent location / customer residence distance is not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Agent location / customer residence distance is not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L204" s="29" t="inlineStr">
@@ -22044,7 +22004,7 @@
       </c>
       <c r="M204" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N204" s="29" t="inlineStr">
@@ -22121,7 +22081,7 @@
       </c>
       <c r="M205" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N205" s="29" t="n"/>
@@ -22194,7 +22154,7 @@
       </c>
       <c r="M206" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N206" s="29" t="n"/>
@@ -22267,7 +22227,7 @@
       </c>
       <c r="M207" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N207" s="29" t="n"/>
@@ -22340,7 +22300,7 @@
       </c>
       <c r="M208" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N208" s="29" t="n"/>
@@ -22413,7 +22373,7 @@
       </c>
       <c r="M209" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N209" s="29" t="n"/>
@@ -22486,7 +22446,7 @@
       </c>
       <c r="M210" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N210" s="29" t="n"/>
@@ -22549,7 +22509,7 @@
       </c>
       <c r="K211" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Rules cannot read links between payers and the merchant owner. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'ownerLinkedPayers'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Rules cannot read links between payers and the merchant owner. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'ownerLinkedPayers'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L211" s="29" t="inlineStr">
@@ -22559,7 +22519,7 @@
       </c>
       <c r="M211" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N211" s="29" t="inlineStr">
@@ -22626,7 +22586,7 @@
       </c>
       <c r="K212" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Rules cannot read links between payers and the merchant owner. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'ownerLinkedPayers'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Rules cannot read links between payers and the merchant owner. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'ownerLinkedPayers'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L212" s="29" t="inlineStr">
@@ -22636,7 +22596,7 @@
       </c>
       <c r="M212" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N212" s="29" t="inlineStr">
@@ -22703,7 +22663,7 @@
       </c>
       <c r="K213" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No sequence pattern 'payment followed by refund or merchant cash-out ≥ P%' scoped to the same merchant (rapidMovement measures any outflow after any inflow, without refund pairing). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'paymentThenRefundShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No sequence pattern 'payment followed by refund or merchant cash-out ≥ P%' scoped to the same merchant (rapidMovement measures any outflow after any inflow, without refund pairing). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'paymentThenRefundShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L213" s="29" t="inlineStr">
@@ -22713,7 +22673,7 @@
       </c>
       <c r="M213" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N213" s="29" t="inlineStr">
@@ -22780,7 +22740,7 @@
       </c>
       <c r="K214" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No sequence pattern 'payment followed by refund or merchant cash-out ≥ P%' scoped to the same merchant (rapidMovement measures any outflow after any inflow, without refund pairing). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'paymentThenRefundShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No sequence pattern 'payment followed by refund or merchant cash-out ≥ P%' scoped to the same merchant (rapidMovement measures any outflow after any inflow, without refund pairing). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'paymentThenRefundShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L214" s="29" t="inlineStr">
@@ -22790,7 +22750,7 @@
       </c>
       <c r="M214" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N214" s="29" t="inlineStr">
@@ -22857,7 +22817,7 @@
       </c>
       <c r="K215" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — POS geolocation and merchant registered area are not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'posDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — POS geolocation and merchant registered area are not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'posDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L215" s="29" t="inlineStr">
@@ -22867,7 +22827,7 @@
       </c>
       <c r="M215" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N215" s="29" t="inlineStr">
@@ -22934,7 +22894,7 @@
       </c>
       <c r="K216" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — POS geolocation and merchant registered area are not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'posDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — POS geolocation and merchant registered area are not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'posDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L216" s="29" t="inlineStr">
@@ -22944,7 +22904,7 @@
       </c>
       <c r="M216" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N216" s="29" t="inlineStr">
@@ -23021,7 +22981,7 @@
       </c>
       <c r="M217" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N217" s="29" t="n"/>
@@ -23094,7 +23054,7 @@
       </c>
       <c r="M218" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N218" s="29" t="n"/>
@@ -23167,7 +23127,7 @@
       </c>
       <c r="M219" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N219" s="29" t="n"/>
@@ -23240,7 +23200,7 @@
       </c>
       <c r="M220" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N220" s="29" t="inlineStr">
@@ -23317,7 +23277,7 @@
       </c>
       <c r="M221" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N221" s="29" t="inlineStr">
@@ -23384,7 +23344,7 @@
       </c>
       <c r="K222" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No sequence pattern of failed attempts with decreasing amounts followed by a success. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'failedDecreasingThenSuccess'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No sequence pattern of failed attempts with decreasing amounts followed by a success. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'failedDecreasingThenSuccess'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L222" s="29" t="inlineStr">
@@ -23394,7 +23354,7 @@
       </c>
       <c r="M222" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N222" s="29" t="inlineStr">
@@ -23461,7 +23421,7 @@
       </c>
       <c r="K223" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No sequence pattern of failed attempts with decreasing amounts followed by a success. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'failedDecreasingThenSuccess'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No sequence pattern of failed attempts with decreasing amounts followed by a success. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'failedDecreasingThenSuccess'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L223" s="29" t="inlineStr">
@@ -23471,7 +23431,7 @@
       </c>
       <c r="M223" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N223" s="29" t="inlineStr">
@@ -23548,7 +23508,7 @@
       </c>
       <c r="M224" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N224" s="29" t="n"/>
@@ -23621,7 +23581,7 @@
       </c>
       <c r="M225" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N225" s="29" t="n"/>
@@ -23684,7 +23644,7 @@
       </c>
       <c r="K226" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Invoice amounts and refund-to-third-party linkage are not captured. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'txn.invoiceAmount': not present in the data-source registry..</t>
+          <t>Capability gap — Invoice amounts are captured (txn.invoiceAmount), but a refund cannot be linked to the third party that receives it, so refunds to third parties cannot be compared with the invoice. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'txn.refundToThirdParty': not present in the data-source registry..</t>
         </is>
       </c>
       <c r="L226" s="29" t="inlineStr">
@@ -23694,7 +23654,7 @@
       </c>
       <c r="M226" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N226" s="29" t="inlineStr">
@@ -23704,7 +23664,7 @@
       </c>
       <c r="O226" s="29" t="inlineStr">
         <is>
-          <t>Automated: Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: invoiceAmount), "···, attempt: { condition = { field = "txn.refundToThirdParty", operator = "eq", value = True }, window = { days = 30, type = "Rolling" } }) (rule validator evidence)</t>
         </is>
       </c>
     </row>
@@ -23761,7 +23721,7 @@
       </c>
       <c r="K227" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Invoice amounts and refund-to-third-party linkage are not captured. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'txn.invoiceAmount': not present in the data-source registry..</t>
+          <t>Capability gap — Invoice amounts are captured (txn.invoiceAmount), but a refund cannot be linked to the third party that receives it, so refunds to third parties cannot be compared with the invoice. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'txn.refundToThirdParty': not present in the data-source registry..</t>
         </is>
       </c>
       <c r="L227" s="29" t="inlineStr">
@@ -23771,7 +23731,7 @@
       </c>
       <c r="M227" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N227" s="29" t="inlineStr">
@@ -23781,7 +23741,7 @@
       </c>
       <c r="O227" s="29" t="inlineStr">
         <is>
-          <t>Automated: Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: invoiceAmount), "···, attempt: { condition = { field = "txn.refundToThirdParty", operator = "eq", value = True }, window = { days = 30, type = "Rolling" } }) (rule validator evidence)</t>
         </is>
       </c>
     </row>
@@ -23848,7 +23808,7 @@
       </c>
       <c r="M228" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N228" s="29" t="n"/>
@@ -23921,7 +23881,7 @@
       </c>
       <c r="M229" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N229" s="29" t="n"/>
@@ -23994,7 +23954,7 @@
       </c>
       <c r="M230" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N230" s="29" t="n"/>
@@ -24067,7 +24027,7 @@
       </c>
       <c r="M231" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N231" s="29" t="n"/>
@@ -24140,7 +24100,7 @@
       </c>
       <c r="M232" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N232" s="29" t="n"/>
@@ -24213,7 +24173,7 @@
       </c>
       <c r="M233" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N233" s="29" t="n"/>
@@ -24286,7 +24246,7 @@
       </c>
       <c r="M234" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N234" s="29" t="n"/>
@@ -24359,7 +24319,7 @@
       </c>
       <c r="M235" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N235" s="29" t="n"/>
@@ -24432,7 +24392,7 @@
       </c>
       <c r="M236" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N236" s="29" t="n"/>
@@ -24505,7 +24465,7 @@
       </c>
       <c r="M237" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N237" s="29" t="n"/>
@@ -24578,7 +24538,7 @@
       </c>
       <c r="M238" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N238" s="29" t="n"/>
@@ -24651,7 +24611,7 @@
       </c>
       <c r="M239" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N239" s="29" t="n"/>
@@ -24724,7 +24684,7 @@
       </c>
       <c r="M240" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N240" s="29" t="n"/>
@@ -24797,7 +24757,7 @@
       </c>
       <c r="M241" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N241" s="29" t="n"/>
@@ -24870,7 +24830,7 @@
       </c>
       <c r="M242" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N242" s="29" t="n"/>
@@ -24943,7 +24903,7 @@
       </c>
       <c r="M243" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N243" s="29" t="n"/>
@@ -25016,7 +24976,7 @@
       </c>
       <c r="M244" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N244" s="29" t="n"/>
@@ -25089,7 +25049,7 @@
       </c>
       <c r="M245" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N245" s="29" t="n"/>
@@ -25162,7 +25122,7 @@
       </c>
       <c r="M246" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N246" s="29" t="n"/>
@@ -25235,7 +25195,7 @@
       </c>
       <c r="M247" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N247" s="29" t="n"/>
@@ -25298,7 +25258,7 @@
       </c>
       <c r="K248" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No corridor share per peer group (nationality/segment). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'corridorPeerShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No corridor share per peer group (nationality/segment). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'corridorPeerShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L248" s="29" t="inlineStr">
@@ -25308,7 +25268,7 @@
       </c>
       <c r="M248" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N248" s="29" t="inlineStr">
@@ -25375,7 +25335,7 @@
       </c>
       <c r="K249" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — No corridor share per peer group (nationality/segment). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'corridorPeerShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No corridor share per peer group (nationality/segment). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'corridorPeerShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="L249" s="29" t="inlineStr">
@@ -25385,7 +25345,7 @@
       </c>
       <c r="M249" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N249" s="29" t="inlineStr">
@@ -25462,7 +25422,7 @@
       </c>
       <c r="M250" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N250" s="29" t="n"/>
@@ -25535,7 +25495,7 @@
       </c>
       <c r="M251" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N251" s="29" t="n"/>
@@ -25608,7 +25568,7 @@
       </c>
       <c r="M252" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N252" s="29" t="n"/>
@@ -25681,7 +25641,7 @@
       </c>
       <c r="M253" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N253" s="29" t="n"/>
@@ -25754,7 +25714,7 @@
       </c>
       <c r="M254" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N254" s="29" t="n"/>
@@ -25827,7 +25787,7 @@
       </c>
       <c r="M255" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N255" s="29" t="n"/>
@@ -25900,7 +25860,7 @@
       </c>
       <c r="M256" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N256" s="29" t="n"/>
@@ -25973,7 +25933,7 @@
       </c>
       <c r="M257" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N257" s="29" t="n"/>
@@ -26046,7 +26006,7 @@
       </c>
       <c r="M258" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N258" s="29" t="n"/>
@@ -26119,7 +26079,7 @@
       </c>
       <c r="M259" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N259" s="29" t="n"/>
@@ -26192,7 +26152,7 @@
       </c>
       <c r="M260" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N260" s="29" t="n"/>
@@ -26265,7 +26225,7 @@
       </c>
       <c r="M261" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N261" s="29" t="n"/>
@@ -26338,7 +26298,7 @@
       </c>
       <c r="M262" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N262" s="29" t="n"/>
@@ -26411,7 +26371,7 @@
       </c>
       <c r="M263" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N263" s="29" t="n"/>
@@ -26484,7 +26444,7 @@
       </c>
       <c r="M264" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N264" s="29" t="n"/>
@@ -26557,7 +26517,7 @@
       </c>
       <c r="M265" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N265" s="29" t="n"/>
@@ -26630,7 +26590,7 @@
       </c>
       <c r="M266" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N266" s="29" t="n"/>
@@ -26703,7 +26663,7 @@
       </c>
       <c r="M267" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N267" s="29" t="n"/>
@@ -26759,14 +26719,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J268" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J268" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K268" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Balances are not available (withdrawal of ≥ P% of balance) and dormancy cannot be combined with a cross-border step sequence. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'wallet.balanceWithdrawnPct': not present in the data-source registry..</t>
+          <t>Dormant 7 months, withdraws 3,700 of a 4,000 balance (92.5 %) and remits abroad within 2 days → 1 alert.</t>
         </is>
       </c>
       <c r="L268" s="29" t="inlineStr">
@@ -26776,17 +26736,13 @@
       </c>
       <c r="M268" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N268" s="29" t="inlineStr">
-        <is>
-          <t>GAP-TF-04</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N268" s="29" t="n"/>
       <c r="O268" s="29" t="inlineStr">
         <is>
-          <t>Automated: Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.TF_04_liquidation_before_travel. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -26836,14 +26792,14 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="J269" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J269" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K269" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Balances are not available (withdrawal of ≥ P% of balance) and dormancy cannot be combined with a cross-border step sequence. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'wallet.balanceWithdrawnPct': not present in the data-source registry..</t>
+          <t>Partial withdrawal (1,500 of 4,000) then remittance → 0 alerts.</t>
         </is>
       </c>
       <c r="L269" s="29" t="inlineStr">
@@ -26853,17 +26809,13 @@
       </c>
       <c r="M269" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N269" s="29" t="inlineStr">
-        <is>
-          <t>GAP-TF-04</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N269" s="29" t="n"/>
       <c r="O269" s="29" t="inlineStr">
         <is>
-          <t>Automated: Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.TF_04_liquidation_before_travel. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -26930,7 +26882,7 @@
       </c>
       <c r="M270" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N270" s="29" t="inlineStr">
@@ -26940,7 +26892,7 @@
       </c>
       <c r="O270" s="29" t="inlineStr">
         <is>
-          <t>Automated: TerroristFinancingSanctionsTests.SAN_01_name_match. Note: the score reached the reject threshold (0.95), so the decision is Reject rather than Hold; a score between 0.85 and 0.95 gives Hold.. Failed in the first execution (DEF-TM-07: Real-time list hits created no AML alert); fixed: Real-time list matches raise Critical/High alerts; re-tested 2026-10-15.</t>
+          <t>Automated: TerroristFinancingSanctionsTests.SAN_01_name_match. Note: the score reached the reject threshold (0.95), so the decision is Reject rather than Hold; a score between 0.85 and 0.95 gives Hold.. Failed in the first execution (DEF-TM-07: Real-time list hits created no AML alert); fixed: Real-time list matches raise Critical/High alerts; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -27007,7 +26959,7 @@
       </c>
       <c r="M271" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N271" s="29" t="n"/>
@@ -27080,7 +27032,7 @@
       </c>
       <c r="M272" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N272" s="29" t="n"/>
@@ -27153,7 +27105,7 @@
       </c>
       <c r="M273" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N273" s="29" t="n"/>
@@ -27226,7 +27178,7 @@
       </c>
       <c r="M274" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N274" s="29" t="n"/>
@@ -27299,7 +27251,7 @@
       </c>
       <c r="M275" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N275" s="29" t="inlineStr">
@@ -27309,7 +27261,7 @@
       </c>
       <c r="O275" s="29" t="inlineStr">
         <is>
-          <t>Automated: TerroristFinancingSanctionsTests.SAN_02_remarks_keywords. Failed in the first execution (DEF-TM-08: Keyword matching without normalisation); fixed: contains normalises case, diacritics and letter spacing; re-tested 2026-10-15.</t>
+          <t>Automated: TerroristFinancingSanctionsTests.SAN_02_remarks_keywords. Failed in the first execution (DEF-TM-08: Keyword matching without normalisation); fixed: contains normalises case, diacritics and letter spacing; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -27376,7 +27328,7 @@
       </c>
       <c r="M276" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N276" s="29" t="n"/>
@@ -27449,7 +27401,7 @@
       </c>
       <c r="M277" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N277" s="29" t="n"/>
@@ -27522,7 +27474,7 @@
       </c>
       <c r="M278" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N278" s="29" t="inlineStr">
@@ -27532,7 +27484,7 @@
       </c>
       <c r="O278" s="29" t="inlineStr">
         <is>
-          <t>Automated: TerroristFinancingSanctionsTests.SAN_04_internal_watchlist. Failed in the first execution (DEF-TM-07: Real-time list hits created no AML alert); fixed: Real-time list matches raise Critical/High alerts; re-tested 2026-10-15.</t>
+          <t>Automated: TerroristFinancingSanctionsTests.SAN_04_internal_watchlist. Failed in the first execution (DEF-TM-07: Real-time list hits created no AML alert); fixed: Real-time list matches raise Critical/High alerts; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -27599,7 +27551,7 @@
       </c>
       <c r="M279" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N279" s="29" t="n"/>
@@ -27655,14 +27607,14 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J280" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J280" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K280" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Password-reset events can be ingested as signals, but wallet balances are not, so 'outgoing ≥ P% of balance' cannot be evaluated. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'event.passwordResetHoursAgo': not present in the data-source registry..</t>
+          <t>Password reset 21:00; 900 of a 1,000 balance (90 %) sent at 21:20 → 1 alert (reset time in the evidence).</t>
         </is>
       </c>
       <c r="L280" s="29" t="inlineStr">
@@ -27672,17 +27624,13 @@
       </c>
       <c r="M280" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N280" s="29" t="inlineStr">
-        <is>
-          <t>GAP-ATO-01</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N280" s="29" t="n"/>
       <c r="O280" s="29" t="inlineStr">
         <is>
-          <t>Automated: Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.ATO_01_password_reset_then_balance_transfer. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -27732,14 +27680,14 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J281" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J281" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K281" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Password-reset events can be ingested as signals, but wallet balances are not, so 'outgoing ≥ P% of balance' cannot be evaluated. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'event.passwordResetHoursAgo': not present in the data-source registry..</t>
+          <t>Reset, no transfer → 0 alerts.</t>
         </is>
       </c>
       <c r="L281" s="29" t="inlineStr">
@@ -27749,17 +27697,13 @@
       </c>
       <c r="M281" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N281" s="29" t="inlineStr">
-        <is>
-          <t>GAP-ATO-01</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N281" s="29" t="n"/>
       <c r="O281" s="29" t="inlineStr">
         <is>
-          <t>Automated: Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.ATO_01_password_reset_then_balance_transfer. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -27809,14 +27753,14 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J282" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J282" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K282" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Beneficiary-added events can be ingested as signals, but wallet balances are not, so 'transfer ≥ P% of balance' cannot be evaluated. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'event.beneficiaryAddedMinutesAgo': not present in the data-source registry..</t>
+          <t>Beneficiary added 10:00; 1,900 of a 2,000 balance (95 %) sent at 10:05 → 1 alert.</t>
         </is>
       </c>
       <c r="L282" s="29" t="inlineStr">
@@ -27826,17 +27770,13 @@
       </c>
       <c r="M282" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N282" s="29" t="inlineStr">
-        <is>
-          <t>GAP-ATO-02</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N282" s="29" t="n"/>
       <c r="O282" s="29" t="inlineStr">
         <is>
-          <t>Automated: Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.ATO_02_new_beneficiary_full_balance_transfer. Note: signals do not identify the beneficiary, so the rule tests the most recent beneficiary addition.. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -27886,14 +27826,14 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="J283" s="30" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="J283" s="28" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="K283" s="29" t="inlineStr">
         <is>
-          <t>Capability gap — Beneficiary-added events can be ingested as signals, but wallet balances are not, so 'transfer ≥ P% of balance' cannot be evaluated. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'event.beneficiaryAddedMinutesAgo': not present in the data-source registry..</t>
+          <t>Long-standing beneficiary (added months earlier) → 0 alerts.</t>
         </is>
       </c>
       <c r="L283" s="29" t="inlineStr">
@@ -27903,17 +27843,13 @@
       </c>
       <c r="M283" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="N283" s="29" t="inlineStr">
-        <is>
-          <t>GAP-ATO-02</t>
-        </is>
-      </c>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="N283" s="29" t="n"/>
       <c r="O283" s="29" t="inlineStr">
         <is>
-          <t>Automated: Scenario_not_configurable (rule validator evidence)</t>
+          <t>Automated: BalanceChainPeerScenarioTests.ATO_02_new_beneficiary_full_balance_transfer. Blocked in earlier executions (capability gap); executable after the balance / chain / peer-percentile extension.</t>
         </is>
       </c>
     </row>
@@ -27980,7 +27916,7 @@
       </c>
       <c r="M284" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N284" s="29" t="n"/>
@@ -28053,7 +27989,7 @@
       </c>
       <c r="M285" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N285" s="29" t="n"/>
@@ -28126,7 +28062,7 @@
       </c>
       <c r="M286" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N286" s="29" t="n"/>
@@ -28199,7 +28135,7 @@
       </c>
       <c r="M287" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N287" s="29" t="n"/>
@@ -28272,7 +28208,7 @@
       </c>
       <c r="M288" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N288" s="29" t="n"/>
@@ -28345,7 +28281,7 @@
       </c>
       <c r="M289" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N289" s="29" t="n"/>
@@ -28418,7 +28354,7 @@
       </c>
       <c r="M290" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N290" s="29" t="n"/>
@@ -28491,7 +28427,7 @@
       </c>
       <c r="M291" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N291" s="29" t="n"/>
@@ -28564,7 +28500,7 @@
       </c>
       <c r="M292" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N292" s="29" t="n"/>
@@ -28637,7 +28573,7 @@
       </c>
       <c r="M293" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N293" s="29" t="n"/>
@@ -28710,7 +28646,7 @@
       </c>
       <c r="M294" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N294" s="29" t="n"/>
@@ -28783,7 +28719,7 @@
       </c>
       <c r="M295" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N295" s="29" t="n"/>
@@ -28856,7 +28792,7 @@
       </c>
       <c r="M296" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N296" s="29" t="n"/>
@@ -28929,7 +28865,7 @@
       </c>
       <c r="M297" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N297" s="29" t="inlineStr">
@@ -28939,7 +28875,7 @@
       </c>
       <c r="O297" s="29" t="inlineStr">
         <is>
-          <t>Automated: EngineEdgeCaseTests.ENG_02_reversal_netting. Failed in the first execution (DEF-TM-09: Later reversal not noted on the alert); fixed: LinkedTransactionReversed entry in alert history; re-tested 2026-10-15.</t>
+          <t>Automated: EngineEdgeCaseTests.ENG_02_reversal_netting. Failed in the first execution (DEF-TM-09: Later reversal not noted on the alert); fixed: LinkedTransactionReversed entry in alert history; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -29006,7 +28942,7 @@
       </c>
       <c r="M298" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N298" s="29" t="n"/>
@@ -29079,7 +29015,7 @@
       </c>
       <c r="M299" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N299" s="29" t="n"/>
@@ -29152,7 +29088,7 @@
       </c>
       <c r="M300" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N300" s="29" t="n"/>
@@ -29225,7 +29161,7 @@
       </c>
       <c r="M301" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N301" s="29" t="n"/>
@@ -29298,7 +29234,7 @@
       </c>
       <c r="M302" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N302" s="29" t="n"/>
@@ -29371,7 +29307,7 @@
       </c>
       <c r="M303" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N303" s="29" t="n"/>
@@ -29444,7 +29380,7 @@
       </c>
       <c r="M304" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N304" s="29" t="inlineStr">
@@ -29454,7 +29390,7 @@
       </c>
       <c r="O304" s="29" t="inlineStr">
         <is>
-          <t>Automated: EngineEdgeCaseTests.ENG_06_late_arrivals. Failed in the first execution (DEF-TM-10: Late arrivals never re-evaluated / not logged); fixed: Scheduler re-evaluates late arrivals within Rules:LateArrivalLookbackDays; older ones raise LateArrivalNotEvaluated; re-tested 2026-10-15.</t>
+          <t>Automated: EngineEdgeCaseTests.ENG_06_late_arrivals. Failed in the first execution (DEF-TM-10: Late arrivals never re-evaluated / not logged); fixed: Scheduler re-evaluates late arrivals within Rules:LateArrivalLookbackDays; older ones raise LateArrivalNotEvaluated; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -29511,7 +29447,7 @@
       </c>
       <c r="K305" s="29" t="inlineStr">
         <is>
-          <t>Transaction dated 40 days ago arriving after its window was evaluated (lookback 7 days, setting Rules:LateArrivalLookbackDays) → data-quality item LateArrivalNotEvaluated: "CORE/E06-OLD-22 dated 2026-09-05T21:29:57.1560308Z arrived after its monitoring window was evaluated and is older than the 7-day re-evaluation lookback; not evaluated by scheduled rules." (visible in the data-quality queue).</t>
+          <t>Transaction dated 40 days ago arriving after its window was evaluated (lookback 7 days, setting Rules:LateArrivalLookbackDays) → data-quality item LateArrivalNotEvaluated: "CORE/E06-OLD-175 dated 2026-09-06T13:14:32.4344729Z arrived after its monitoring window was evaluated and is older than the 7-day re-evaluation lookback; not evaluated by scheduled rules." (visible in the data-quality queue).</t>
         </is>
       </c>
       <c r="L305" s="29" t="inlineStr">
@@ -29521,7 +29457,7 @@
       </c>
       <c r="M305" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N305" s="29" t="inlineStr">
@@ -29531,7 +29467,7 @@
       </c>
       <c r="O305" s="29" t="inlineStr">
         <is>
-          <t>Automated: EngineEdgeCaseTests.ENG_06_late_arrivals. Failed in the first execution (DEF-TM-10: Late arrivals never re-evaluated / not logged); fixed: Scheduler re-evaluates late arrivals within Rules:LateArrivalLookbackDays; older ones raise LateArrivalNotEvaluated; re-tested 2026-10-15.</t>
+          <t>Automated: EngineEdgeCaseTests.ENG_06_late_arrivals. Failed in the first execution (DEF-TM-10: Late arrivals never re-evaluated / not logged); fixed: Scheduler re-evaluates late arrivals within Rules:LateArrivalLookbackDays; older ones raise LateArrivalNotEvaluated; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -29598,7 +29534,7 @@
       </c>
       <c r="M306" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N306" s="29" t="inlineStr">
@@ -29608,7 +29544,7 @@
       </c>
       <c r="O306" s="29" t="inlineStr">
         <is>
-          <t>Automated: EngineEdgeCaseTests.ENG_07_customer_vs_wallet_level. Failed in the first execution (DEF-TM-11: No wallet-level aggregation; unresolved parties not evaluated); fixed: Subject 'Wallet' and unresolvedParties = Wallet; re-tested 2026-10-15.</t>
+          <t>Automated: EngineEdgeCaseTests.ENG_07_customer_vs_wallet_level. Failed in the first execution (DEF-TM-11: No wallet-level aggregation; unresolved parties not evaluated); fixed: Subject 'Wallet' and unresolvedParties = Wallet; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -29665,7 +29601,7 @@
       </c>
       <c r="K307" s="29" t="inlineStr">
         <is>
-          <t>20 withdrawals from an unresolved wallet → 2 UnresolvedParty data-quality item; customer rule with unresolvedParties = Wallet evaluates the wallet itself → 1 wallet-level alert (subject wallet:W-UNRESOLVED-34b03d).</t>
+          <t>20 withdrawals from an unresolved wallet → 2 UnresolvedParty data-quality item; customer rule with unresolvedParties = Wallet evaluates the wallet itself → 1 wallet-level alert (subject wallet:W-UNRESOLVED-c4ab8d).</t>
         </is>
       </c>
       <c r="L307" s="29" t="inlineStr">
@@ -29675,7 +29611,7 @@
       </c>
       <c r="M307" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N307" s="29" t="inlineStr">
@@ -29685,7 +29621,7 @@
       </c>
       <c r="O307" s="29" t="inlineStr">
         <is>
-          <t>Automated: EngineEdgeCaseTests.ENG_07_customer_vs_wallet_level. Failed in the first execution (DEF-TM-11: No wallet-level aggregation; unresolved parties not evaluated); fixed: Subject 'Wallet' and unresolvedParties = Wallet; re-tested 2026-10-15.</t>
+          <t>Automated: EngineEdgeCaseTests.ENG_07_customer_vs_wallet_level. Failed in the first execution (DEF-TM-11: No wallet-level aggregation; unresolved parties not evaluated); fixed: Subject 'Wallet' and unresolvedParties = Wallet; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -29752,7 +29688,7 @@
       </c>
       <c r="M308" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N308" s="29" t="n"/>
@@ -29825,7 +29761,7 @@
       </c>
       <c r="M309" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N309" s="29" t="n"/>
@@ -29898,7 +29834,7 @@
       </c>
       <c r="M310" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N310" s="29" t="n"/>
@@ -29971,7 +29907,7 @@
       </c>
       <c r="M311" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N311" s="29" t="n"/>
@@ -30044,7 +29980,7 @@
       </c>
       <c r="M312" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N312" s="29" t="inlineStr">
@@ -30054,7 +29990,7 @@
       </c>
       <c r="O312" s="29" t="inlineStr">
         <is>
-          <t>Automated: EngineEdgeCaseTests.ENG_10_fees_and_clearing. Failed in the first execution (DEF-TM-12: Clearing-wallet legs double counted); fixed: Second leg marked EconomicLegOfId and excluded from monitoring/aggregates; re-tested 2026-10-15.</t>
+          <t>Automated: EngineEdgeCaseTests.ENG_10_fees_and_clearing. Failed in the first execution (DEF-TM-12: Clearing-wallet legs double counted); fixed: Second leg marked EconomicLegOfId and excluded from monitoring/aggregates; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -30121,7 +30057,7 @@
       </c>
       <c r="M313" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N313" s="29" t="inlineStr">
@@ -30131,7 +30067,7 @@
       </c>
       <c r="O313" s="29" t="inlineStr">
         <is>
-          <t>Automated: EngineEdgeCaseTests.ENG_11_realtime_batch_consistency. Failed in the first execution (DEF-TM-13: Real-time holds not linked to batch alerts); fixed: Real-time rule hits raise the alert with the batch deduplication key; re-tested 2026-10-15.</t>
+          <t>Automated: EngineEdgeCaseTests.ENG_11_realtime_batch_consistency. Failed in the first execution (DEF-TM-13: Real-time holds not linked to batch alerts); fixed: Real-time rule hits raise the alert with the batch deduplication key; re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -30198,7 +30134,7 @@
       </c>
       <c r="M314" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N314" s="29" t="inlineStr">
@@ -30265,7 +30201,7 @@
       </c>
       <c r="K315" s="29" t="inlineStr">
         <is>
-          <t>Customer with 50,000 transactions in one calendar-month window (200 ingested through the API in 14 s, the rest cloned in SQL): synchronous rule run completed in 8.4 s with 1 alert.</t>
+          <t>Customer with 50,000 transactions in one calendar-month window (200 ingested through the API in 13 s, the rest cloned in SQL): synchronous rule run completed in 12.7 s with 1 alert.</t>
         </is>
       </c>
       <c r="L315" s="29" t="inlineStr">
@@ -30275,7 +30211,7 @@
       </c>
       <c r="M315" s="29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="N315" s="29" t="inlineStr">
@@ -30285,7 +30221,7 @@
       </c>
       <c r="O315" s="29" t="inlineStr">
         <is>
-          <t>Automated: EngineScaleTests.ENG_12_scale. Failed in the first execution (DEF-TM-14: Quadratic rule evaluation (50k transactions did not finish)); fixed: Indexed windows, prefix sums, deferred evidence, merge by dedup key (50k in ~10 s); re-tested 2026-10-15.</t>
+          <t>Automated: EngineScaleTests.ENG_12_scale. Failed in the first execution (DEF-TM-14: Quadratic rule evaluation (50k transactions did not finish)); fixed: Indexed windows, prefix sums, deferred evidence, merge by dedup key (50k in ~10 s); re-tested 2026-10-16.</t>
         </is>
       </c>
     </row>
@@ -30477,7 +30413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="16" min="1" max="1"/>
@@ -30829,7 +30765,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Capability gap — Rules cannot test links between the agent and the customers it serves (shared ID/phone/device/family). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentLinkedCustomerTxns'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Rules cannot test links between the agent and the customers it serves (shared ID/phone/device/family). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentLinkedCustomerTxns'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -30851,7 +30787,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Capability gap — peerRatio uses agent volume, not the cash-out/cash-in ratio compared with a regional peer median × R. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerRatioOfRatio'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — peerRatio uses agent volume, not the cash-out/cash-in ratio compared with a regional peer median × R. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerRatioOfRatio'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -30873,7 +30809,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Capability gap — No 'customers registered by agent who transact within 24 h' share aggregate. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentNewCustomerActiveShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No 'customers registered by agent who transact within 24 h' share aggregate. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentNewCustomerActiveShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -30895,7 +30831,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Capability gap — Agent location / customer residence distance is not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Agent location / customer residence distance is not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -30907,7 +30843,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GAP-AMT-06</t>
+          <t>GAP-BEH-07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -30917,19 +30853,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Capability gap — peerRatio compares with the peer median of agent-processed volume only; no percentile, segment or minimum peer-group size. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'peerPercentile'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No salary-credit linkage or 'M consecutive months' pattern. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'salaryRemittedShareConsecutiveMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>TM-AMT-06-01, TM-AMT-06-02, TM-AMT-06-03</t>
+          <t>TM-BEH-07-01, TM-BEH-07-02</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GAP-ATO-01</t>
+          <t>GAP-DEV-03</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -30939,19 +30875,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Capability gap — Password-reset events can be ingested as signals, but wallet balances are not, so 'outgoing ≥ P% of balance' cannot be evaluated. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'event.passwordResetHoursAgo': not present in the data-source registry..</t>
+          <t>Capability gap — IP anonymiser (VPN/proxy/TOR) classification is not captured or exposed to rules. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'session.ipAnonymiser': not present in the data-source registry..</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TM-ATO-01-01, TM-ATO-01-02</t>
+          <t>TM-DEV-03-01, TM-DEV-03-02</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GAP-ATO-02</t>
+          <t>GAP-DEV-04</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -30961,19 +30897,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Capability gap — Beneficiary-added events can be ingested as signals, but wallet balances are not, so 'transfer ≥ P% of balance' cannot be evaluated. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'event.beneficiaryAddedMinutesAgo': not present in the data-source registry..</t>
+          <t>Capability gap — Rooted/jailbroken/emulator device flags are not captured or exposed to rules. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'device.rooted': not present in the data-source registry..</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>TM-ATO-02-01, TM-ATO-02-02</t>
+          <t>TM-DEV-04-01, TM-DEV-04-02</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>GAP-BEH-07</t>
+          <t>GAP-DEV-07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -30983,19 +30919,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Capability gap — No salary-credit linkage or 'M consecutive months' pattern. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'salaryRemittedShareConsecutiveMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Channel limit-hit events are not ingested; channel switch sequence cannot be expressed. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'channelSwitchAfterLimit'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>TM-BEH-07-01, TM-BEH-07-02</t>
+          <t>TM-DEV-07-01, TM-DEV-07-02</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>GAP-DEV-03</t>
+          <t>GAP-GEO-01</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -31005,19 +30941,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Capability gap — IP anonymiser (VPN/proxy/TOR) classification is not captured or exposed to rules. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'session.ipAnonymiser': not present in the data-source registry..</t>
+          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>TM-DEV-03-01, TM-DEV-03-02</t>
+          <t>TM-GEO-01-01, TM-GEO-01-02, TM-GEO-01-03, TM-GEO-01-04, TM-GEO-01-05</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>GAP-DEV-04</t>
+          <t>GAP-GEO-07</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -31027,19 +30963,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Capability gap — Rooted/jailbroken/emulator device flags are not captured or exposed to rules. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'device.rooted': not present in the data-source registry..</t>
+          <t>Capability gap — No 'first cross-border after M months domestic-only' aggregate (newCountries ignores amount and months of domestic history). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'firstCrossBorderAfterMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>TM-DEV-04-01, TM-DEV-04-02</t>
+          <t>TM-GEO-07-01, TM-GEO-07-02</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GAP-DEV-07</t>
+          <t>GAP-GEO-08</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -31049,19 +30985,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Capability gap — Channel limit-hit events are not ingested; channel switch sequence cannot be expressed. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'channelSwitchAfterLimit'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Agent locations / distances are not modelled; cash-in and cash-out by different persons cannot be correlated. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TM-DEV-07-01, TM-DEV-07-02</t>
+          <t>TM-GEO-08-01, TM-GEO-08-02</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GAP-GEO-01</t>
+          <t>GAP-GEO-09</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -31071,19 +31007,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Capability gap — No geolocation or distance/speed (impossible travel) computation; transactions carry country only. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'travelSpeedKmh'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No border-zone agent classification available to rules (agent attributes are not readable from customer-subject rules). Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'agent.borderZone': not present in the data-source registry..</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>TM-GEO-01-01, TM-GEO-01-02, TM-GEO-01-03, TM-GEO-01-04, TM-GEO-01-05</t>
+          <t>TM-GEO-09-01, TM-GEO-09-02</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GAP-GEO-07</t>
+          <t>GAP-MER-03</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -31093,19 +31029,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Capability gap — No 'first cross-border after M months domestic-only' aggregate (newCountries ignores amount and months of domestic history). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'firstCrossBorderAfterMonths'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Rules cannot read links between payers and the merchant owner. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'ownerLinkedPayers'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>TM-GEO-07-01, TM-GEO-07-02</t>
+          <t>TM-MER-03-01, TM-MER-03-02</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GAP-GEO-08</t>
+          <t>GAP-MER-04</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -31115,19 +31051,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Capability gap — Agent locations / distances are not modelled; cash-in and cash-out by different persons cannot be correlated. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'agentDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No sequence pattern 'payment followed by refund or merchant cash-out ≥ P%' scoped to the same merchant (rapidMovement measures any outflow after any inflow, without refund pairing). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'paymentThenRefundShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>TM-GEO-08-01, TM-GEO-08-02</t>
+          <t>TM-MER-04-01, TM-MER-04-02</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GAP-GEO-09</t>
+          <t>GAP-MER-05</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -31137,19 +31073,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Capability gap — No border-zone agent classification available to rules (agent attributes are not readable from customer-subject rules). Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'agent.borderZone': not present in the data-source registry..</t>
+          <t>Capability gap — POS geolocation and merchant registered area are not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'posDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>TM-GEO-09-01, TM-GEO-09-02</t>
+          <t>TM-MER-05-01, TM-MER-05-02</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GAP-MER-03</t>
+          <t>GAP-REV-02</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -31159,19 +31095,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Capability gap — Rules cannot read links between payers and the merchant owner. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'ownerLinkedPayers'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Refund destination instrument vs original payment instrument is not captured. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'txn.refundInstrumentMismatch': not present in the data-source registry..</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>TM-MER-03-01, TM-MER-03-02</t>
+          <t>TM-REV-02-01, TM-REV-02-02</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GAP-MER-04</t>
+          <t>GAP-REV-03</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -31181,19 +31117,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Capability gap — No sequence pattern 'payment followed by refund or merchant cash-out ≥ P%' scoped to the same merchant (rapidMovement measures any outflow after any inflow, without refund pairing). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'paymentThenRefundShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No sequence pattern of failed attempts with decreasing amounts followed by a success. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'failedDecreasingThenSuccess'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>TM-MER-04-01, TM-MER-04-02</t>
+          <t>TM-REV-03-01, TM-REV-03-02</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>GAP-MER-05</t>
+          <t>GAP-REV-05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -31203,19 +31139,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Capability gap — POS geolocation and merchant registered area are not modelled. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'posDistanceKm'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — Invoice amounts are captured (txn.invoiceAmount), but a refund cannot be linked to the third party that receives it, so refunds to third parties cannot be compared with the invoice. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'txn.refundToThirdParty': not present in the data-source registry..</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>TM-MER-05-01, TM-MER-05-02</t>
+          <t>TM-REV-05-01, TM-REV-05-02</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GAP-REV-02</t>
+          <t>GAP-VEL-07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -31225,19 +31161,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Capability gap — Refund destination instrument vs original payment instrument is not captured. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'txn.refundInstrumentMismatch': not present in the data-source registry..</t>
+          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>TM-REV-02-01, TM-REV-02-02</t>
+          <t>TM-VEL-07-01, TM-VEL-07-02, TM-VEL-07-03, TM-VEL-07-04</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GAP-REV-03</t>
+          <t>GAP-XBR-03</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -31247,142 +31183,10 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Capability gap — No sequence pattern of failed attempts with decreasing amounts followed by a success. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'failedDecreasingThenSuccess'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
+          <t>Capability gap — No corridor share per peer group (nationality/segment). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'corridorPeerShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent, avgBalance, minBalance, balanceRetentionPct, chain, peerPercentile, benchmarkDeviation..</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
-        <is>
-          <t>TM-REV-03-01, TM-REV-03-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>GAP-REV-05</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Capability gap (test cases Blocked)</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Capability gap — Invoice amounts and refund-to-third-party linkage are not captured. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'txn.invoiceAmount': not present in the data-source registry..</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>TM-REV-05-01, TM-REV-05-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>GAP-RMV-02</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Capability gap (test cases Blocked)</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Capability gap — Wallet balances / end-of-day balances are not ingested or available to rules. Closest rule definition rejected by the rule validator: $.condition.conditions[0].field: Unknown field 'wallet.endOfDayBalance': not present in the data-source registry..</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>TM-RMV-02-01, TM-RMV-02-02, TM-RMV-02-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>GAP-RMV-04</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Capability gap (test cases Blocked)</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Capability gap — cycle detects funds returning to the subject only; no open multi-hop chain (A→B→C→D) with per-hop retention. Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'chain'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>TM-RMV-04-01, TM-RMV-04-02, TM-RMV-04-03, TM-RMV-04-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>GAP-TF-04</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Capability gap (test cases Blocked)</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Capability gap — Balances are not available (withdrawal of ≥ P% of balance) and dormancy cannot be combined with a cross-border step sequence. Closest rule definition rejected by the rule validator: $.condition.field: Unknown field 'wallet.balanceWithdrawnPct': not present in the data-source registry..</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>TM-TF-04-01, TM-TF-04-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>GAP-VEL-07</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Capability gap (test cases Blocked)</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Capability gap — No aggregate for regularity of time gaps (standard deviation of inter-transaction intervals). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'intervalStdDev'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>TM-VEL-07-01, TM-VEL-07-02, TM-VEL-07-03, TM-VEL-07-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>GAP-XBR-03</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Capability gap (test cases Blocked)</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Capability gap — No corridor share per peer group (nationality/segment). Closest rule definition rejected by the rule validator: $.condition.aggregate: Unknown aggregate 'corridorPeerShare'. Allowed: count, sum, distinctCounterparties, ratio, rapidMovement, dormancyDays, profileRatio, peerRatio, newCustomers, customersPerDevice, cycle, newCountries, historyCount, historySum, historyRatio, distinctCount, reciprocalCount, consecutiveDays, newCounterpartyShare, sharedDeviceSenders, typeShareChange, minutesSinceEvent..</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
         <is>
           <t>TM-XBR-03-01, TM-XBR-03-02</t>
         </is>

</xml_diff>